<commit_message>
Replace two-check schedule with rotating 5-slot coverage roster
Confirmed ustraveldocs.com's Terms of Service prohibit automated
bots/scripts checking slot availability, so instead of 24/7 automation
the team covers 5 check windows/day (9:30, 11:30, 1:30, 3:30, 5:30) on a
rotating roster across all 8 agents — closes the "nobody's watching"
gap without violating the portal's ToS or risking a client's booked
appointment getting access-limited.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DiEcNy7XAwqHLRjhRBareN
</commit_message>
<xml_diff>
--- a/trackers/US_VISA_SLOT_WATCH_LOG.xlsx
+++ b/trackers/US_VISA_SLOT_WATCH_LOG.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Slot Watch Log" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Pattern Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Coverage Roster" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,8 +56,18 @@
       <b val="1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF0000FF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF808080"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +77,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E2F3"/>
       </patternFill>
     </fill>
   </fills>
@@ -81,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -99,6 +115,16 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -532,7 +558,7 @@
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="B3:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"9:00 AM,3:00 PM,Other"</formula1>
+      <formula1>"9:30 AM,11:30 AM,1:30 PM,3:30 PM,5:30 PM,Other"</formula1>
     </dataValidation>
     <dataValidation sqref="D3:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Abu Dhabi,Dubai"</formula1>
@@ -551,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -606,7 +632,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>9:00 AM</t>
+          <t>9:30 AM</t>
         </is>
       </c>
       <c r="B6" s="6">
@@ -625,7 +651,7 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>3:00 PM</t>
+          <t>11:30 AM</t>
         </is>
       </c>
       <c r="B7" s="6">
@@ -644,7 +670,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>1:30 PM</t>
         </is>
       </c>
       <c r="B8" s="6">
@@ -660,80 +686,137 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>3:30 PM</t>
+        </is>
+      </c>
+      <c r="B9" s="6">
+        <f>COUNTIF('Slot Watch Log'!$B$3:$B$200,A9)</f>
+        <v/>
+      </c>
+      <c r="C9" s="6">
+        <f>COUNTIFS('Slot Watch Log'!$B$3:$B$200,A9,'Slot Watch Log'!$F$3:$F$200,"Yes")</f>
+        <v/>
+      </c>
+      <c r="D9" s="7">
+        <f>IFERROR(C9/B9,0)</f>
+        <v/>
+      </c>
+    </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="B10" s="6">
+        <f>COUNTIF('Slot Watch Log'!$B$3:$B$200,A10)</f>
+        <v/>
+      </c>
+      <c r="C10" s="6">
+        <f>COUNTIFS('Slot Watch Log'!$B$3:$B$200,A10,'Slot Watch Log'!$F$3:$F$200,"Yes")</f>
+        <v/>
+      </c>
+      <c r="D10" s="7">
+        <f>IFERROR(C10/B10,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B11" s="6">
+        <f>COUNTIF('Slot Watch Log'!$B$3:$B$200,A11)</f>
+        <v/>
+      </c>
+      <c r="C11" s="6">
+        <f>COUNTIFS('Slot Watch Log'!$B$3:$B$200,A11,'Slot Watch Log'!$F$3:$F$200,"Yes")</f>
+        <v/>
+      </c>
+      <c r="D11" s="7">
+        <f>IFERROR(C11/B11,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>BY CONSULATE</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>CONSULATE</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>TOTAL CHECKS</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>SLOTS FOUND</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>HIT RATE</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Abu Dhabi</t>
         </is>
       </c>
-      <c r="B12" s="6">
-        <f>COUNTIF('Slot Watch Log'!$D$3:$D$200,A12)</f>
-        <v/>
-      </c>
-      <c r="C12" s="6">
-        <f>COUNTIFS('Slot Watch Log'!$D$3:$D$200,A12,'Slot Watch Log'!$F$3:$F$200,"Yes")</f>
-        <v/>
-      </c>
-      <c r="D12" s="7">
-        <f>IFERROR(C12/B12,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="B15" s="6">
+        <f>COUNTIF('Slot Watch Log'!$D$3:$D$200,A15)</f>
+        <v/>
+      </c>
+      <c r="C15" s="6">
+        <f>COUNTIFS('Slot Watch Log'!$D$3:$D$200,A15,'Slot Watch Log'!$F$3:$F$200,"Yes")</f>
+        <v/>
+      </c>
+      <c r="D15" s="7">
+        <f>IFERROR(C15/B15,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Dubai</t>
         </is>
       </c>
-      <c r="B13" s="6">
-        <f>COUNTIF('Slot Watch Log'!$D$3:$D$200,A13)</f>
-        <v/>
-      </c>
-      <c r="C13" s="6">
-        <f>COUNTIFS('Slot Watch Log'!$D$3:$D$200,A13,'Slot Watch Log'!$F$3:$F$200,"Yes")</f>
-        <v/>
-      </c>
-      <c r="D13" s="7">
-        <f>IFERROR(C13/B13,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="B16" s="6">
+        <f>COUNTIF('Slot Watch Log'!$D$3:$D$200,A16)</f>
+        <v/>
+      </c>
+      <c r="C16" s="6">
+        <f>COUNTIFS('Slot Watch Log'!$D$3:$D$200,A16,'Slot Watch Log'!$F$3:$F$200,"Yes")</f>
+        <v/>
+      </c>
+      <c r="D16" s="7">
+        <f>IFERROR(C16/B16,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>TOTAL LOGGED CHECKS</t>
         </is>
       </c>
-      <c r="B15" s="8">
+      <c r="B18" s="8">
         <f>COUNTA('Slot Watch Log'!$A$3:$A$200)</f>
         <v/>
       </c>
@@ -745,4 +828,276 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25.5" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SLOT-CHECK COVERAGE ROSTER — WEEKLY TEMPLATE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Replaces 24/7 automated monitoring (against ustraveldocs.com's Terms of Service) with human coverage spread across the day. Blue cells = editable — swap names for leave/sick days. Rotation is pre-filled so no single agent carries every shift.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>DAY</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>9:30 AM</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>11:30 AM</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>1:30 PM</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>3:30 PM</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Layan (ATL)</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Ibrahim</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Chaima</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Alshima</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>Saha</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Khosema</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Harinder</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Rihab</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>Layan (ATL)</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>Ibrahim</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Chaima</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Alshima</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Saha</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Khosema</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>Harinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Rihab</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Layan (ATL)</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Ibrahim</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Chaima</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>Alshima</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Saha</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Khosema</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Harinder</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>Rihab</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>Layan (ATL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Ibrahim</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Chaima</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Alshima</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>Saha</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>Khosema</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Sunday: office closed, no checks scheduled. Whoever is on shift logs the result — including “no slots” — in the Slot Watch Log tab straight after checking.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A12:F12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>